<commit_message>
made into light theme
</commit_message>
<xml_diff>
--- a/backend/sample_feedback.xlsx
+++ b/backend/sample_feedback.xlsx
@@ -425,715 +425,1430 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A101"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>feedback</t>
+          <t>Feedback Id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Content Id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Feedback Text</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Reply Text</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>2982</v>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>The platform is well-designed and I had no issues whatsoever.</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>5061</v>
+      </c>
+      <c r="C3" t="inlineStr">
         <is>
           <t>The platform is well-designed and I had no issues whatsoever.</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4681</v>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>I was unable to submit my answers due to a technical error.</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2049</v>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Very poor performance. The page took forever to load each question.</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6539</v>
+      </c>
+      <c r="C6" t="inlineStr">
         <is>
           <t>I really appreciate how stable the system was during the entire exam.</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1344</v>
+      </c>
+      <c r="C7" t="inlineStr">
         <is>
           <t>The timer malfunctioned and I lost precious time. Unacceptable!</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>4770</v>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>The system logged me out mid-exam for no reason whatsoever.</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>4608</v>
+      </c>
+      <c r="C9" t="inlineStr">
         <is>
           <t>The UI is very confusing. I could not find the submit button.</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1117</v>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>The timer malfunctioned and I lost precious time. Unacceptable!</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2163</v>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>Some features felt outdated but the core functionality was fine.</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1964</v>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>4750</v>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>The experience was neither exceptional nor terrible. Just normal.</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>2104</v>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>My answers were not saved and I had to retype everything again.</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1514</v>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>6413</v>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>The exam portal worked flawlessly throughout the session.</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>2160</v>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>Had to refresh once but everything was alright after that.</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>9423</v>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>Great experience! The interface is very user-friendly and intuitive.</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>4899</v>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>The server response was fantastic, no lag at all. Great work!</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>5562</v>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t>Loved the clean UI. Everything was straightforward and easy to navigate.</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>8953</v>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>My answers were not saved and I had to retype everything again.</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4510</v>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>9834</v>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>Decent portal. Could be improved with a better mobile experience.</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>3167</v>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>Superb performance. I completed my exam without any interruption.</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>8744</v>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>4981</v>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>Decent portal. Could be improved with a better mobile experience.</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>8749</v>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>Excellent system support! The exam was a great experience overall.</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>7669</v>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>Excellent system support! The exam was a great experience overall.</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4119</v>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>The exam portal worked flawlessly throughout the session.</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>2545</v>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>Average experience. Some sections worked fine, others had minor lag.</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>2588</v>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>Very poor performance. The page took forever to load each question.</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>8062</v>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>6804</v>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>7939</v>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>Some features felt outdated but the core functionality was fine.</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>7735</v>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>The page kept freezing and I lost my progress multiple times.</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>8651</v>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>The server response was fantastic, no lag at all. Great work!</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>1887</v>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>It was alright. The interface is basic but functional enough.</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>2612</v>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>It was alright. The interface is basic but functional enough.</t>
         </is>
       </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1993</v>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>The exam completed without major issues but had occasional slowness.</t>
         </is>
       </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>7596</v>
+      </c>
+      <c r="C40" t="inlineStr">
         <is>
           <t>Terrible experience. The system crashed twice during the test.</t>
         </is>
       </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>6559</v>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>Terrible experience. The system crashed twice during the test.</t>
         </is>
       </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>2790</v>
+      </c>
+      <c r="C42" t="inlineStr">
         <is>
           <t>Decent portal. Could be improved with a better mobile experience.</t>
         </is>
       </c>
+      <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>5073</v>
+      </c>
+      <c r="C43" t="inlineStr">
         <is>
           <t>The page kept freezing and I lost my progress multiple times.</t>
         </is>
       </c>
+      <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>4139</v>
+      </c>
+      <c r="C44" t="inlineStr">
         <is>
           <t>The UI is very confusing. I could not find the submit button.</t>
         </is>
       </c>
+      <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4116</v>
+      </c>
+      <c r="C45" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>9786</v>
+      </c>
+      <c r="C46" t="inlineStr">
         <is>
           <t>Superb performance. I completed my exam without any interruption.</t>
         </is>
       </c>
+      <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>8350</v>
+      </c>
+      <c r="C47" t="inlineStr">
         <is>
           <t>The exam portal worked flawlessly throughout the session.</t>
         </is>
       </c>
+      <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>3296</v>
+      </c>
+      <c r="C48" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>7912</v>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>Could not access the exam at all. Server was down the whole time.</t>
         </is>
       </c>
+      <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>4006</v>
+      </c>
+      <c r="C50" t="inlineStr">
         <is>
           <t>The timer malfunctioned and I lost precious time. Unacceptable!</t>
         </is>
       </c>
+      <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>5563</v>
+      </c>
+      <c r="C51" t="inlineStr">
         <is>
           <t>The system worked as expected. Nothing remarkable to report.</t>
         </is>
       </c>
+      <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>8579</v>
+      </c>
+      <c r="C52" t="inlineStr">
         <is>
           <t>Could not access the exam at all. Server was down the whole time.</t>
         </is>
       </c>
+      <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>5092</v>
+      </c>
+      <c r="C53" t="inlineStr">
         <is>
           <t>The exam completed without major issues but had occasional slowness.</t>
         </is>
       </c>
+      <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>2235</v>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>The system worked as expected. Nothing remarkable to report.</t>
         </is>
       </c>
+      <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>8260</v>
+      </c>
+      <c r="C55" t="inlineStr">
         <is>
           <t>The exam was okay. Nothing special but nothing terrible either.</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>2604</v>
+      </c>
+      <c r="C56" t="inlineStr">
         <is>
           <t>The exam completed without major issues but had occasional slowness.</t>
         </is>
       </c>
+      <c r="D56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1828</v>
+      </c>
+      <c r="C57" t="inlineStr">
         <is>
           <t>Very poor performance. The page took forever to load each question.</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>9856</v>
+      </c>
+      <c r="C58" t="inlineStr">
         <is>
           <t>The server response was fantastic, no lag at all. Great work!</t>
         </is>
       </c>
+      <c r="D58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>1241</v>
+      </c>
+      <c r="C59" t="inlineStr">
         <is>
           <t>The system worked as expected. Nothing remarkable to report.</t>
         </is>
       </c>
+      <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>2528</v>
+      </c>
+      <c r="C60" t="inlineStr">
         <is>
           <t>The server went down in the middle of my exam. Very frustrating!</t>
         </is>
       </c>
+      <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>4872</v>
+      </c>
+      <c r="C61" t="inlineStr">
         <is>
           <t>The exam completed without major issues but had occasional slowness.</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>3724</v>
+      </c>
+      <c r="C62" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="n">
+        <v>7658</v>
+      </c>
+      <c r="C63" t="inlineStr">
         <is>
           <t>I really appreciate how stable the system was during the entire exam.</t>
         </is>
       </c>
+      <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="n">
+        <v>8956</v>
+      </c>
+      <c r="C64" t="inlineStr">
         <is>
           <t>I really appreciate how stable the system was during the entire exam.</t>
         </is>
       </c>
+      <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="n">
+        <v>8886</v>
+      </c>
+      <c r="C65" t="inlineStr">
         <is>
           <t>I was unable to submit my answers due to a technical error.</t>
         </is>
       </c>
+      <c r="D65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="n">
+        <v>4502</v>
+      </c>
+      <c r="C66" t="inlineStr">
         <is>
           <t>I really appreciate how stable the system was during the entire exam.</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="n">
+        <v>7570</v>
+      </c>
+      <c r="C67" t="inlineStr">
         <is>
           <t>Terrible experience. The system crashed twice during the test.</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1960</v>
+      </c>
+      <c r="C68" t="inlineStr">
         <is>
           <t>The server went down in the middle of my exam. Very frustrating!</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="n">
+        <v>3697</v>
+      </c>
+      <c r="C69" t="inlineStr">
         <is>
           <t>The platform is well-designed and I had no issues whatsoever.</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="n">
+        <v>7209</v>
+      </c>
+      <c r="C70" t="inlineStr">
         <is>
           <t>Had to refresh once but everything was alright after that.</t>
         </is>
       </c>
+      <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1035</v>
+      </c>
+      <c r="C71" t="inlineStr">
         <is>
           <t>The exam was okay. Nothing special but nothing terrible either.</t>
         </is>
       </c>
+      <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="n">
+        <v>7396</v>
+      </c>
+      <c r="C72" t="inlineStr">
         <is>
           <t>The exam portal worked flawlessly throughout the session.</t>
         </is>
       </c>
+      <c r="D72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="n">
+        <v>5345</v>
+      </c>
+      <c r="C73" t="inlineStr">
         <is>
           <t>The timer malfunctioned and I lost precious time. Unacceptable!</t>
         </is>
       </c>
+      <c r="D73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="n">
+        <v>8454</v>
+      </c>
+      <c r="C74" t="inlineStr">
         <is>
           <t>Great experience! The interface is very user-friendly and intuitive.</t>
         </is>
       </c>
+      <c r="D74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="n">
+        <v>5673</v>
+      </c>
+      <c r="C75" t="inlineStr">
         <is>
           <t>Could not access the exam at all. Server was down the whole time.</t>
         </is>
       </c>
+      <c r="D75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="n">
+        <v>7930</v>
+      </c>
+      <c r="C76" t="inlineStr">
         <is>
           <t>I was unable to submit my answers due to a technical error.</t>
         </is>
       </c>
+      <c r="D76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="n">
+        <v>8973</v>
+      </c>
+      <c r="C77" t="inlineStr">
         <is>
           <t>I was unable to submit my answers due to a technical error.</t>
         </is>
       </c>
+      <c r="D77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="n">
+        <v>3536</v>
+      </c>
+      <c r="C78" t="inlineStr">
         <is>
           <t>The system logged me out mid-exam for no reason whatsoever.</t>
         </is>
       </c>
+      <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="n">
+        <v>4111</v>
+      </c>
+      <c r="C79" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D79" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="n">
+        <v>5861</v>
+      </c>
+      <c r="C80" t="inlineStr">
         <is>
           <t>It was alright. The interface is basic but functional enough.</t>
         </is>
       </c>
+      <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="n">
+        <v>4566</v>
+      </c>
+      <c r="C81" t="inlineStr">
         <is>
           <t>The exam completed without major issues but had occasional slowness.</t>
         </is>
       </c>
+      <c r="D81" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="n">
+        <v>1958</v>
+      </c>
+      <c r="C82" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="n">
+        <v>9883</v>
+      </c>
+      <c r="C83" t="inlineStr">
         <is>
           <t>Not bad, not great. The exam process was standard.</t>
         </is>
       </c>
+      <c r="D83" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="n">
+        <v>1998</v>
+      </c>
+      <c r="C84" t="inlineStr">
         <is>
           <t>The server response was fantastic, no lag at all. Great work!</t>
         </is>
       </c>
+      <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="n">
+        <v>6138</v>
+      </c>
+      <c r="C85" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="n">
+        <v>1936</v>
+      </c>
+      <c r="C86" t="inlineStr">
         <is>
           <t>I'm impressed by the smooth performance and quick load times.</t>
         </is>
       </c>
+      <c r="D86" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="n">
+        <v>1821</v>
+      </c>
+      <c r="C87" t="inlineStr">
         <is>
           <t>The exam portal worked flawlessly throughout the session.</t>
         </is>
       </c>
+      <c r="D87" t="inlineStr"/>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="n">
+        <v>8811</v>
+      </c>
+      <c r="C88" t="inlineStr">
         <is>
           <t>The timer malfunctioned and I lost precious time. Unacceptable!</t>
         </is>
       </c>
+      <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="n">
+        <v>9238</v>
+      </c>
+      <c r="C89" t="inlineStr">
         <is>
           <t>Could not access the exam at all. Server was down the whole time.</t>
         </is>
       </c>
+      <c r="D89" t="inlineStr"/>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="n">
+        <v>9701</v>
+      </c>
+      <c r="C90" t="inlineStr">
         <is>
           <t>Superb performance. I completed my exam without any interruption.</t>
         </is>
       </c>
+      <c r="D90" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="n">
+        <v>3579</v>
+      </c>
+      <c r="C91" t="inlineStr">
         <is>
           <t>Great experience! The interface is very user-friendly and intuitive.</t>
         </is>
       </c>
+      <c r="D91" t="inlineStr"/>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="n">
+        <v>1931</v>
+      </c>
+      <c r="C92" t="inlineStr">
         <is>
           <t>I was unable to submit my answers due to a technical error.</t>
         </is>
       </c>
+      <c r="D92" t="inlineStr"/>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="n">
+        <v>9320</v>
+      </c>
+      <c r="C93" t="inlineStr">
         <is>
           <t>Very poor performance. The page took forever to load each question.</t>
         </is>
       </c>
+      <c r="D93" t="inlineStr"/>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="n">
+        <v>2312</v>
+      </c>
+      <c r="C94" t="inlineStr">
         <is>
           <t>Had to refresh once but everything was alright after that.</t>
         </is>
       </c>
+      <c r="D94" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="n">
+        <v>4044</v>
+      </c>
+      <c r="C95" t="inlineStr">
         <is>
           <t>Terrible experience. The system crashed twice during the test.</t>
         </is>
       </c>
+      <c r="D95" t="inlineStr"/>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="n">
+        <v>2122</v>
+      </c>
+      <c r="C96" t="inlineStr">
         <is>
           <t>The system logged me out mid-exam for no reason whatsoever.</t>
         </is>
       </c>
+      <c r="D96" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="n">
+        <v>2113</v>
+      </c>
+      <c r="C97" t="inlineStr">
         <is>
           <t>The timer was accurate and the submission went smoothly.</t>
         </is>
       </c>
+      <c r="D97" t="inlineStr"/>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="n">
+        <v>4853</v>
+      </c>
+      <c r="C98" t="inlineStr">
         <is>
           <t>Could not access the exam at all. Server was down the whole time.</t>
         </is>
       </c>
+      <c r="D98" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="n">
+        <v>7615</v>
+      </c>
+      <c r="C99" t="inlineStr">
         <is>
           <t>I was unable to submit my answers due to a technical error.</t>
         </is>
       </c>
+      <c r="D99" t="inlineStr"/>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="n">
+        <v>2964</v>
+      </c>
+      <c r="C100" t="inlineStr">
         <is>
           <t>Some features felt outdated but the core functionality was fine.</t>
         </is>
       </c>
+      <c r="D100" t="inlineStr"/>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="n">
+        <v>5033</v>
+      </c>
+      <c r="C101" t="inlineStr">
         <is>
           <t>Excellent system support! The exam was a great experience overall.</t>
         </is>
       </c>
+      <c r="D101" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>